<commit_message>
Recompute the fixed-regimen contrast and correct the exposure description
76/6,167 versus 7/1,098, rate ratio 1.93 (0.89-4.18): direction unchanged, interval includes unity, so the within-class claim is softened. Exposure is described as the drugname/prod_ai single-token match that was actually used.
</commit_message>
<xml_diff>
--- a/submission/Supplementary_Tables.xlsx
+++ b/submission/Supplementary_Tables.xlsx
@@ -1024,7 +1024,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E8"/>
+  <dimension ref="A1:E9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1196,18 +1196,39 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>5736</v>
+        <v>6167</v>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>3.24 (rate ratio)</t>
+          <t>1.93 (rate ratio)</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>1.02-10.28</t>
-        </is>
-      </c>
+          <t>0.89-4.18</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Fixed regimen: RIF+INH+PZA without ethambutol</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Optic-nerve event, rate ratio (reference)</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>1098</v>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>reference</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Second review round: period coverage, regimen in main_results, figure labels, release tag
57 pre-2004 cases now account for the period split. The fixed-regimen contrast is exported in main_results.json. Figure 3 and Table 4 separate negative controls from non-specific comparators. PROGRESS.md carries the current numbers.
</commit_message>
<xml_diff>
--- a/submission/Supplementary_Tables.xlsx
+++ b/submission/Supplementary_Tables.xlsx
@@ -13,6 +13,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="S4_canada" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="S5_flow" sheetId="5" state="visible" r:id="rId5"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="S6_zero_cells" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="S7_period_coverage" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -476,217 +477,217 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Vision blurred</t>
+          <t>Cataract</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>control</t>
+          <t>negative control</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>151</v>
+        <v>39</v>
       </c>
       <c r="D2" t="n">
-        <v>135063</v>
+        <v>58616</v>
       </c>
       <c r="E2" t="n">
-        <v>1.5</v>
+        <v>0.89</v>
       </c>
       <c r="F2" t="n">
-        <v>1.28</v>
+        <v>0.65</v>
       </c>
       <c r="G2" t="n">
-        <v>1.76</v>
+        <v>1.22</v>
       </c>
       <c r="H2" t="n">
-        <v>1.035233624816228e-06</v>
+        <v>0.4775214192246711</v>
       </c>
       <c r="I2" t="n">
-        <v>112</v>
+        <v>26</v>
       </c>
       <c r="J2" t="n">
-        <v>1.91</v>
+        <v>1.02</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Cataract</t>
+          <t>Conjunctivitis</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>control</t>
+          <t>negative control</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>39</v>
+        <v>11</v>
       </c>
       <c r="D3" t="n">
-        <v>58616</v>
+        <v>18170</v>
       </c>
       <c r="E3" t="n">
-        <v>0.89</v>
+        <v>0.8100000000000001</v>
       </c>
       <c r="F3" t="n">
-        <v>0.65</v>
+        <v>0.45</v>
       </c>
       <c r="G3" t="n">
-        <v>1.22</v>
+        <v>1.46</v>
       </c>
       <c r="H3" t="n">
         <v>0.4775214192246711</v>
       </c>
       <c r="I3" t="n">
-        <v>26</v>
+        <v>5</v>
       </c>
       <c r="J3" t="n">
-        <v>1.02</v>
+        <v>0.63</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Conjunctivitis</t>
+          <t>Dry eye</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>control</t>
+          <t>negative control</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D4" t="n">
-        <v>18170</v>
+        <v>47855</v>
       </c>
       <c r="E4" t="n">
-        <v>0.8100000000000001</v>
+        <v>0.28</v>
       </c>
       <c r="F4" t="n">
-        <v>0.45</v>
+        <v>0.15</v>
       </c>
       <c r="G4" t="n">
-        <v>1.46</v>
+        <v>0.52</v>
       </c>
       <c r="H4" t="n">
-        <v>0.4775214192246711</v>
+        <v>2.070398277041042e-05</v>
       </c>
       <c r="I4" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="J4" t="n">
-        <v>0.63</v>
+        <v>0.33</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Eye pain</t>
+          <t>Glaucoma</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>control</t>
+          <t>negative control</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>27</v>
+        <v>4</v>
       </c>
       <c r="D5" t="n">
-        <v>54555</v>
+        <v>19045</v>
       </c>
       <c r="E5" t="n">
-        <v>0.66</v>
+        <v>0.28</v>
       </c>
       <c r="F5" t="n">
-        <v>0.45</v>
+        <v>0.11</v>
       </c>
       <c r="G5" t="n">
-        <v>0.96</v>
+        <v>0.75</v>
       </c>
       <c r="H5" t="n">
-        <v>0.03410167056764134</v>
+        <v>0.008115896832008505</v>
       </c>
       <c r="I5" t="n">
-        <v>16</v>
+        <v>2</v>
       </c>
       <c r="J5" t="n">
-        <v>0.67</v>
+        <v>0.24</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Dry eye</t>
+          <t>Vision blurred</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>control</t>
+          <t>non-specific comparator</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>10</v>
+        <v>151</v>
       </c>
       <c r="D6" t="n">
-        <v>47855</v>
+        <v>135063</v>
       </c>
       <c r="E6" t="n">
-        <v>0.28</v>
+        <v>1.5</v>
       </c>
       <c r="F6" t="n">
-        <v>0.15</v>
+        <v>1.28</v>
       </c>
       <c r="G6" t="n">
-        <v>0.52</v>
+        <v>1.76</v>
       </c>
       <c r="H6" t="n">
-        <v>2.070398277041042e-05</v>
+        <v>1.035233624816228e-06</v>
       </c>
       <c r="I6" t="n">
-        <v>7</v>
+        <v>112</v>
       </c>
       <c r="J6" t="n">
-        <v>0.33</v>
+        <v>1.91</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Glaucoma</t>
+          <t>Eye pain</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>control</t>
+          <t>non-specific comparator</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>4</v>
+        <v>27</v>
       </c>
       <c r="D7" t="n">
-        <v>19045</v>
+        <v>54555</v>
       </c>
       <c r="E7" t="n">
-        <v>0.28</v>
+        <v>0.66</v>
       </c>
       <c r="F7" t="n">
-        <v>0.11</v>
+        <v>0.45</v>
       </c>
       <c r="G7" t="n">
-        <v>0.75</v>
+        <v>0.96</v>
       </c>
       <c r="H7" t="n">
-        <v>0.008115896832008505</v>
+        <v>0.03410167056764134</v>
       </c>
       <c r="I7" t="n">
-        <v>2</v>
+        <v>16</v>
       </c>
       <c r="J7" t="n">
-        <v>0.24</v>
+        <v>0.67</v>
       </c>
     </row>
     <row r="8">
@@ -2604,4 +2605,60 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Item</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>De-duplicated cases</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>20692683</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Cases with at least one receipt date in 2004-2026</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>20692626</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Cases whose every receipt date precedes 2004 (outside both periods)</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>57</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Third review round: replication boundary, composite outcome, onset sample, q formatting
Cross-system replication now applies to the optic-nerve signal only; Canada Vigilance does not support a term-level control comparison. The fixed-regimen outcome is defined as a four-term composite and reported as a ratio of reporting proportions. The onset analysis reports its sample sizes and missingness, and explains its wider 17-term definition. q values that underflow are displayed as <1e-300.
</commit_message>
<xml_diff>
--- a/submission/Supplementary_Tables.xlsx
+++ b/submission/Supplementary_Tables.xlsx
@@ -14,6 +14,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="S5_flow" sheetId="5" state="visible" r:id="rId5"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="S6_zero_cells" sheetId="6" state="visible" r:id="rId6"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="S7_period_coverage" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="S8_onset_sample" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="S9_onset_terms" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -500,8 +502,10 @@
       <c r="G2" t="n">
         <v>1.22</v>
       </c>
-      <c r="H2" t="n">
-        <v>0.4775214192246711</v>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>0.4775</t>
+        </is>
       </c>
       <c r="I2" t="n">
         <v>26</v>
@@ -536,8 +540,10 @@
       <c r="G3" t="n">
         <v>1.46</v>
       </c>
-      <c r="H3" t="n">
-        <v>0.4775214192246711</v>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>0.4775</t>
+        </is>
       </c>
       <c r="I3" t="n">
         <v>5</v>
@@ -572,8 +578,10 @@
       <c r="G4" t="n">
         <v>0.52</v>
       </c>
-      <c r="H4" t="n">
-        <v>2.070398277041042e-05</v>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>2.1e-05</t>
+        </is>
       </c>
       <c r="I4" t="n">
         <v>7</v>
@@ -608,8 +616,10 @@
       <c r="G5" t="n">
         <v>0.75</v>
       </c>
-      <c r="H5" t="n">
-        <v>0.008115896832008505</v>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>0.008116</t>
+        </is>
       </c>
       <c r="I5" t="n">
         <v>2</v>
@@ -644,8 +654,10 @@
       <c r="G6" t="n">
         <v>1.76</v>
       </c>
-      <c r="H6" t="n">
-        <v>1.035233624816228e-06</v>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>1.0e-06</t>
+        </is>
       </c>
       <c r="I6" t="n">
         <v>112</v>
@@ -680,8 +692,10 @@
       <c r="G7" t="n">
         <v>0.96</v>
       </c>
-      <c r="H7" t="n">
-        <v>0.03410167056764134</v>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>0.0341</t>
+        </is>
       </c>
       <c r="I7" t="n">
         <v>16</v>
@@ -716,8 +730,10 @@
       <c r="G8" t="n">
         <v>304.56</v>
       </c>
-      <c r="H8" t="n">
-        <v>0</v>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>&lt;1e-300</t>
+        </is>
       </c>
       <c r="I8" t="n">
         <v>35</v>
@@ -752,8 +768,10 @@
       <c r="G9" t="n">
         <v>607.55</v>
       </c>
-      <c r="H9" t="n">
-        <v>1.157971571074784e-104</v>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>1.2e-104</t>
+        </is>
       </c>
       <c r="I9" t="n">
         <v>3</v>
@@ -788,8 +806,10 @@
       <c r="G10" t="n">
         <v>136.78</v>
       </c>
-      <c r="H10" t="n">
-        <v>0</v>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>&lt;1e-300</t>
+        </is>
       </c>
       <c r="I10" t="n">
         <v>157</v>
@@ -824,8 +844,10 @@
       <c r="G11" t="n">
         <v>95.18000000000001</v>
       </c>
-      <c r="H11" t="n">
-        <v>1.942829586319284e-19</v>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>1.9e-19</t>
+        </is>
       </c>
       <c r="I11" t="n">
         <v>2</v>
@@ -860,8 +882,10 @@
       <c r="G12" t="n">
         <v>27.75</v>
       </c>
-      <c r="H12" t="n">
-        <v>0</v>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>&lt;1e-300</t>
+        </is>
       </c>
       <c r="I12" t="n">
         <v>141</v>
@@ -896,8 +920,10 @@
       <c r="G13" t="n">
         <v>29.94</v>
       </c>
-      <c r="H13" t="n">
-        <v>3.297020966761631e-94</v>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>3.3e-94</t>
+        </is>
       </c>
       <c r="I13" t="n">
         <v>23</v>
@@ -932,8 +958,10 @@
       <c r="G14" t="n">
         <v>18.95</v>
       </c>
-      <c r="H14" t="n">
-        <v>1.780541641906212e-14</v>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>1.8e-14</t>
+        </is>
       </c>
       <c r="I14" t="n">
         <v>7</v>
@@ -968,8 +996,10 @@
       <c r="G15" t="n">
         <v>14.68</v>
       </c>
-      <c r="H15" t="n">
-        <v>1.221943344747402e-12</v>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>1.2e-12</t>
+        </is>
       </c>
       <c r="I15" t="n">
         <v>8</v>
@@ -1004,8 +1034,10 @@
       <c r="G16" t="n">
         <v>9.26</v>
       </c>
-      <c r="H16" t="n">
-        <v>2.604845647864022e-19</v>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>2.6e-19</t>
+        </is>
       </c>
       <c r="I16" t="n">
         <v>13</v>
@@ -1193,7 +1225,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Optic-nerve event, rate ratio</t>
+          <t>Optic-nerve composite (4 preferred terms), ratio of reporting proportions</t>
         </is>
       </c>
       <c r="C8" t="n">
@@ -1201,7 +1233,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>1.93 (rate ratio)</t>
+          <t>1.93 (ratio of proportions)</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -2661,4 +2693,270 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D7"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Group</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Analysable interval</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Missing or unusable dates</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>All ethambutol cases</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>15510</v>
+      </c>
+      <c r="C2" t="inlineStr"/>
+      <c r="D2" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Analysable interval (all)</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>2446</v>
+      </c>
+      <c r="C3" t="inlineStr"/>
+      <c r="D3" t="n">
+        <v>13064</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Optic-nerve event</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>83</v>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Any ocular event</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>157</v>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>No ocular event</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>2289</v>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Cases carrying at least one of the 17 optic-nerve terms</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>472</v>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>83</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:A18"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Optic-nerve term used in the onset analysis</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>OPTIC NEUROPATHY</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>OPTIC NEURITIS</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>OPTIC ATROPHY</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>OPTIC NERVE DISORDER</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>OPTIC NERVE INJURY</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>OPTIC DISC DISORDER</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>PAPILLOEDEMA</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>BLINDNESS</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>BLINDNESS UNILATERAL</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>BLINDNESS BILATERAL</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>SUDDEN VISUAL LOSS</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>VISUAL FIELD DEFECT</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>SCOTOMA</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>DYSCHROMATOPSIA</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>CHROMATOPSIA</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>HEMIANOPIA</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>OCULAR TOXICITY</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Fourth review round: control grouping, vision-blurred exception, onset groups, declarations
Results 3.3 now matches the Methods grouping of four negative controls and two non-specific comparators. Discussion 4.3 reports the vision-blurred excess and no longer claims anatomical specificity. The onset section names the other-ocular group and the primary comparison. The abstract separates optic-nerve replication from the control-term comparison. Declarations follow the TADS format with separate items and a Plain Language Title.
</commit_message>
<xml_diff>
--- a/submission/Supplementary_Tables.xlsx
+++ b/submission/Supplementary_Tables.xlsx
@@ -2701,7 +2701,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D7"/>
+  <dimension ref="A1:D8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2771,11 +2771,11 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Any ocular event</t>
+          <t>Other ocular event (neither optic-nerve nor non-ocular)</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>157</v>
+        <v>74</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -2787,11 +2787,11 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>No ocular event</t>
+          <t>Any ocular event</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>2289</v>
+        <v>157</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
@@ -2803,18 +2803,34 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
+          <t>No ocular event</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>2289</v>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
           <t>Cases carrying at least one of the 17 optic-nerve terms</t>
         </is>
       </c>
-      <c r="B7" t="n">
+      <c r="B8" t="n">
         <v>472</v>
       </c>
-      <c r="C7" t="inlineStr">
+      <c r="C8" t="inlineStr">
         <is>
           <t>83</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr"/>
+      <c r="D8" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Separate the Canadian composite from the SMQ, and remove methods promises the supplement does not keep
Canada Vigilance is now an exploratory string-matched composite with its own definition and limitations; the Table 3 footnote distinguishes the 1,308 database-wide reports from exposed reports. The PRR/IC025 and logistic-regression claims are removed, the comparator list is reduced to the three drugs analysed, the onset list is cited as S9, the autophagy wording no longer claims a flux blockade, and the READUS-PV checklist is supplied as a Word file.
</commit_message>
<xml_diff>
--- a/submission/Supplementary_Tables.xlsx
+++ b/submission/Supplementary_Tables.xlsx
@@ -455,7 +455,7 @@
     <col width="10" customWidth="1" min="5" max="5"/>
     <col width="14" customWidth="1" min="6" max="6"/>
     <col width="14" customWidth="1" min="7" max="7"/>
-    <col width="16" customWidth="1" min="8" max="8"/>
+    <col width="11" customWidth="1" min="8" max="8"/>
     <col width="11" customWidth="1" min="9" max="9"/>
     <col width="20" customWidth="1" min="10" max="10"/>
     <col width="29" customWidth="1" min="11" max="11"/>
@@ -508,7 +508,7 @@
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>p (exact test)</t>
+          <t>P value</t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr">
@@ -1902,12 +1902,12 @@
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>Any preferred term containing the string OPTIC</t>
+          <t>Any preferred term containing the string OPTIC (study-specific composite)</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>the MedDRA narrow optic-nerve search is defined as all terms containing 'optic'; the Canadian extract is coded to MedDRA 29.0, so the rule is applied directly</t>
+          <t>this is a string match built for this analysis, not a re-implementation of the 45-term Optic nerve disorders query; it includes terms of different clinical meaning, such as imaging terms and surgical procedures, so the Canadian result is exploratory</t>
         </is>
       </c>
       <c r="C4" s="3" t="n">

</xml_diff>

<commit_message>
Restructure S8, settle the JADER mapping claim, set references in Vancouver style, add a Word manuscript
</commit_message>
<xml_diff>
--- a/submission/Supplementary_Tables.xlsx
+++ b/submission/Supplementary_Tables.xlsx
@@ -1553,13 +1553,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D17"/>
+  <dimension ref="A1:D18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="31" customWidth="1" min="1" max="1"/>
+    <col width="34" customWidth="1" min="1" max="1"/>
     <col width="24" customWidth="1" min="2" max="2"/>
-    <col width="10" customWidth="1" min="3" max="3"/>
-    <col width="41" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="48" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -1844,6 +1844,24 @@
       <c r="D17" s="3" t="inlineStr">
         <is>
           <t>control terms used in the same analysis</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="3" t="inlineStr">
+        <is>
+          <t>(no analysed term failed to map)</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="inlineStr"/>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>not applicable</t>
+        </is>
+      </c>
+      <c r="D18" s="3" t="inlineStr">
+        <is>
+          <t>every analysed term had a Japanese equivalent, so no term was excluded for mapping failure</t>
         </is>
       </c>
     </row>
@@ -4475,13 +4493,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D9"/>
+  <dimension ref="A1:D10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="48" customWidth="1" min="1" max="1"/>
-    <col width="10" customWidth="1" min="2" max="2"/>
-    <col width="21" customWidth="1" min="3" max="3"/>
-    <col width="27" customWidth="1" min="4" max="4"/>
+    <col width="13" customWidth="1" min="2" max="2"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="38" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -4499,17 +4517,17 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>n</t>
+          <t>Total cases</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>Analysable interval</t>
+          <t>Cases with a usable interval</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>Missing or unusable dates</t>
+          <t>Cases with missing or unusable dates</t>
         </is>
       </c>
     </row>
@@ -4522,86 +4540,80 @@
       <c r="B4" s="3" t="n">
         <v>15510</v>
       </c>
-      <c r="C4" s="3" t="inlineStr"/>
-      <c r="D4" s="3" t="inlineStr"/>
+      <c r="C4" s="3" t="n">
+        <v>2446</v>
+      </c>
+      <c r="D4" s="3" t="n">
+        <v>13064</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>Analysable interval (all)</t>
+          <t>Cases carrying at least one of the 17 optic-nerve terms</t>
         </is>
       </c>
       <c r="B5" s="3" t="n">
-        <v>2446</v>
-      </c>
-      <c r="C5" s="3" t="inlineStr"/>
+        <v>472</v>
+      </c>
+      <c r="C5" s="3" t="n">
+        <v>83</v>
+      </c>
       <c r="D5" s="3" t="n">
-        <v>13064</v>
+        <v>389</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="3" t="inlineStr">
-        <is>
-          <t>Optic-nerve event</t>
-        </is>
-      </c>
-      <c r="B6" s="3" t="n">
-        <v>83</v>
-      </c>
-      <c r="C6" s="3" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
+      <c r="A6" s="3" t="inlineStr"/>
+      <c r="B6" s="3" t="inlineStr"/>
+      <c r="C6" s="3" t="inlineStr"/>
       <c r="D6" s="3" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>Other ocular event (neither optic-nerve nor non-ocular)</t>
-        </is>
-      </c>
-      <c r="B7" s="3" t="n">
-        <v>74</v>
-      </c>
-      <c r="C7" s="3" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
+          <t>Composition of the 2,446 cases with a usable interval</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="inlineStr"/>
+      <c r="C7" s="3" t="inlineStr"/>
       <c r="D7" s="3" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
         <is>
-          <t>No ocular event</t>
-        </is>
-      </c>
-      <c r="B8" s="3" t="n">
-        <v>2289</v>
-      </c>
-      <c r="C8" s="3" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
+          <t xml:space="preserve">  optic-nerve event</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="inlineStr"/>
+      <c r="C8" s="3" t="n">
+        <v>83</v>
       </c>
       <c r="D8" s="3" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>Cases carrying at least one of the 17 optic-nerve terms</t>
-        </is>
-      </c>
-      <c r="B9" s="3" t="n">
-        <v>472</v>
-      </c>
-      <c r="C9" s="3" t="inlineStr">
-        <is>
-          <t>83</t>
-        </is>
+          <t xml:space="preserve">  other ocular event</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="inlineStr"/>
+      <c r="C9" s="3" t="n">
+        <v>74</v>
       </c>
       <c r="D9" s="3" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  non-ocular event</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="inlineStr"/>
+      <c r="C10" s="3" t="n">
+        <v>2289</v>
+      </c>
+      <c r="D10" s="3" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>